<commit_message>
fix(map): stop unnecessary refreshing on scroll & improve AI navigation
</commit_message>
<xml_diff>
--- a/excel_data/Hausanschluss_data.xlsx
+++ b/excel_data/Hausanschluss_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESC_LAP_RPA 2\EnergyBot_Offline\excel_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B980EC25-8F45-4E91-ACFD-19D2EB5E9796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA945E1C-C9FC-43AF-BC97-C907C0ABE1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3439,7 +3439,7 @@
   <dimension ref="A1:CF60"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.5546875" bestFit="1" customWidth="1"/>

</xml_diff>